<commit_message>
Mise à jour octobre MTD au 10/10 (extraction 65) : performance mensuelle, zéro achat (section 5.4 MTD), bundle soja-concentrés (section 10 MTD), analyse trend (P1 05-10/10, deux baisses de prix), booster 13 mois, soja octobre (T1-T5)
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/download/analyse_soja_octobre.xlsx
+++ b/download/analyse_soja_octobre.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="T1 - Moy jour soja par agence" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="T2 - Commandes soja 03-10" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="T3 - Soja-only 03-10" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="T2 - Commandes soja 10-10" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="T3 - Soja-only 10-10" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="T4 - Stock soja et rupture" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="T5 - Tendance Octobre" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,10 +47,6 @@
     <font>
       <i val="1"/>
       <color rgb="00375623"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="009C0006"/>
       <sz val="10"/>
     </font>
     <font>
@@ -161,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -170,17 +166,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -305,12 +300,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$A$5:$A$9</f>
+              <f>'T5 - Tendance Octobre'!$A$5:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$D$5:$D$9</f>
+              <f>'T5 - Tendance Octobre'!$D$5:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -340,12 +335,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$A$5:$A$9</f>
+              <f>'T5 - Tendance Octobre'!$A$5:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$E$5:$E$9</f>
+              <f>'T5 - Tendance Octobre'!$E$5:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -452,12 +447,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$A$5:$A$9</f>
+              <f>'T5 - Tendance Octobre'!$A$5:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$G$5:$G$9</f>
+              <f>'T5 - Tendance Octobre'!$G$5:$G$14</f>
             </numRef>
           </val>
         </ser>
@@ -882,7 +877,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>01/10 au 03/10/2026 (3j). Livree. lun-sam. Mise a jour 05/10/2026.</t>
+          <t>01/10 au 10/10/2026 (9j). Livree. lun-sam. Mise a jour 10/10/2026.</t>
         </is>
       </c>
     </row>
@@ -925,14 +920,14 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>155.9</v>
+        <v>710.4</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>52</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>+0.6 t/j</t>
+          <t>+27.5 t/j</t>
         </is>
       </c>
     </row>
@@ -948,14 +943,14 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>100.5</v>
+        <v>362.3</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>33.5</v>
+        <v>40.3</v>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>+12.1 t/j</t>
+          <t>+18.8 t/j</t>
         </is>
       </c>
     </row>
@@ -971,14 +966,14 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>57.4</v>
+        <v>283.1</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>19.1</v>
+        <v>31.5</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>+2.9 t/j</t>
+          <t>+15.3 t/j</t>
         </is>
       </c>
     </row>
@@ -994,14 +989,14 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>53.5</v>
+        <v>194</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>17.8</v>
+        <v>21.6</v>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>+2.6 t/j</t>
+          <t>+6.4 t/j</t>
         </is>
       </c>
     </row>
@@ -1017,21 +1012,21 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>36.6</v>
+        <v>122.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>12.2</v>
+        <v>13.6</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+0.5 t/j</t>
+          <t>+1.9 t/j</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Nkoabang</t>
+          <t>Ahala</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1040,21 +1035,21 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>35.7</v>
+        <v>117.3</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>11.9</v>
+        <v>13</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>+1.7 t/j</t>
+          <t>+2.6 t/j</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Ahala</t>
+          <t>Nkoabang</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1063,60 +1058,60 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>32</v>
+        <v>115.3</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>10.7</v>
+        <v>12.8</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>+0.2 t/j</t>
+          <t>+2.6 t/j</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Mbouda</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>31.6</v>
+        <v>113</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>10.5</v>
+        <v>12.6</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>+1.7 t/j</t>
+          <t>+4.2 t/j</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Mbouda</t>
+          <t>Pk11</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>25.2</v>
+        <v>99</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>+0.1 t/j</t>
+        <v>11</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>+2.2 t/j</t>
         </is>
       </c>
     </row>
@@ -1132,14 +1127,14 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>23.9</v>
+        <v>96</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>8</v>
+        <v>10.7</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>+1.4 t/j</t>
+          <t>+4.1 t/j</t>
         </is>
       </c>
     </row>
@@ -1155,14 +1150,14 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>21.6</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>-0.7 t/j</t>
+        <v>10.1</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>+2.2 t/j</t>
         </is>
       </c>
     </row>
@@ -1178,14 +1173,14 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>20</v>
+        <v>67.5</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>6.7</v>
+        <v>7.5</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>+0.8 t/j</t>
+          <t>+1.6 t/j</t>
         </is>
       </c>
     </row>
@@ -1201,14 +1196,14 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>10.6</v>
+        <v>47.1</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>3.5</v>
+        <v>5.2</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>+1.0 t/j</t>
+          <t>+2.8 t/j</t>
         </is>
       </c>
     </row>
@@ -1224,14 +1219,14 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>5</v>
+        <v>30.8</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>-0.6 t/j</t>
+        <v>3.4</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>+1.1 t/j</t>
         </is>
       </c>
     </row>
@@ -1247,104 +1242,104 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>-0.1 t/j</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>TOTAL Ouest</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Ouest</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>238.6</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>79.5</v>
-      </c>
-      <c r="E20" s="7" t="n"/>
+      <c r="C20" s="6" t="n">
+        <v>1106.4</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>122.9</v>
+      </c>
+      <c r="E20" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>TOTAL Centre</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Centre</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n">
-        <v>158.5</v>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>52.8</v>
-      </c>
-      <c r="E21" s="7" t="n"/>
+      <c r="C21" s="6" t="n">
+        <v>595.4</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="E21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>TOTAL Littoral</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Littoral</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n">
-        <v>212.6</v>
-      </c>
-      <c r="D22" s="7" t="n">
-        <v>70.90000000000001</v>
-      </c>
-      <c r="E22" s="7" t="n"/>
+      <c r="C22" s="6" t="n">
+        <v>747.3</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="E22" s="6" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="8" t="n">
-        <v>610.6</v>
-      </c>
-      <c r="D23" s="8" t="n">
-        <v>203.5</v>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>+24.3 t/j vs 179.3</t>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n">
+        <v>2451.1</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>272.3</v>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>+93.1 t/j vs 179.3</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>NOTE: Prix du soja en septembre 2026: 23 879 FCFA/sac (hausse de +2 000 XAF/sac depuis le 23/07/2026).</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Moyenne/jour globale: 203.5 t/j (4070 sacs) sur 3j.</t>
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Moyenne/jour globale: 272.3 t/j (5446 sacs) sur 9j.</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1353,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Note: extraction du 05/10 — aucune commande Livrée le 04/10 (dimanche) ni le 05/10 (commandes encore Validées/En cours).</t>
+          <t>Note: extraction du 12/10 — commandes Livrées jusqu'au 10/10 (le 11/10 est un dimanche).</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1388,14 +1383,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TABLEAU 2 - Commandes SOJA le 03/10/2026 par agence</t>
+          <t>TABLEAU 2 - Commandes SOJA le 10/10/2026 par agence</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Livree. Ratio en sacs 50kg-equivalent. Mise a jour 05/10/2026.</t>
+          <t>Livree. Ratio en sacs 50kg-equivalent. Mise a jour 10/10/2026.</t>
         </is>
       </c>
     </row>
@@ -1448,29 +1443,29 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>4.3:1</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>-15 cmdes</t>
+          <t>3.9:1</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>-17 cmdes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Ahala</t>
+          <t>Messassi</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1479,10 +1474,10 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>0</v>
@@ -1492,47 +1487,47 @@
           <t>2.6:1</t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>-1 cmdes</t>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>-2 cmdes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Messassi</t>
+          <t>Pk11</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2.4:1</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>-10 cmdes</t>
+          <t>1.7:1</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>-6 cmdes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Village</t>
+          <t>Buea</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1541,65 +1536,65 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>2.6:1</t>
+          <t>3.2:1</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>-3 cmdes</t>
+          <t>+4 cmdes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Mbouda</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>4.8:1</t>
+          <t>1.3:1</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>-6 cmdes</t>
+          <t>+2 cmdes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Buea</t>
+          <t>Nkolbisson</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
@@ -1613,19 +1608,19 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>3.0:1</t>
-        </is>
-      </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>+3 cmdes</t>
+          <t>2.8:1</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>+2 cmdes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Nkoabang</t>
+          <t>Bertoua</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1634,29 +1629,29 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>3.3:1</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>stable</t>
+          <t>1.2:1</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>-11 cmdes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Bertoua</t>
+          <t>Ahala</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1675,19 +1670,19 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>1.9:1</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>-11 cmdes</t>
+          <t>2.5:1</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>-6 cmdes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Mbouda</t>
+          <t>Djeleng</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1696,29 +1691,29 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>1.8:1</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>-3 cmdes</t>
+          <t>2.6:1</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>-9 cmdes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Nkolbisson</t>
+          <t>Nkoabang</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1727,20 +1722,20 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>3.0:1</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="inlineStr">
+          <t>3.6:1</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
         <is>
           <t>-3 cmdes</t>
         </is>
@@ -1758,200 +1753,169 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>4.3:1</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>-5 cmdes</t>
+          <t>1.5:1</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>-6 cmdes</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Ndobo</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Littoral</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>∞</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>-11 cmdes</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n">
-        <v>110</v>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>87</v>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>4.7:1</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>-85 cmdes vs 195</t>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n">
+        <v>111</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>97</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>2.3:1</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>-84 cmdes vs 195</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Distribution ratios (bundle seulement)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>Distribution ratios (bundle seulement)</t>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Tranche</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Nb cmdes</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Part</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Tranche</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Nb cmdes</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Part</t>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>&lt;= 3:1</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>77%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>&lt;= 3:1</t>
+          <t>3-5:1</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>62%</t>
+          <t>19%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>3-5:1</t>
+          <t>5-10:1</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>3%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>5-10:1</t>
+          <t>10-20:1</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>1%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>10-20:1</t>
+          <t>&gt; 20:1</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>&gt; 20:1</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
           <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>NOTE: Prix du soja: 23 879 FCFA/sac en moyenne septembre 2026 ; octobre MTD 19 318 FCFA/sac — baisse du 07/10 (20 500 → 17 600 FCFA/sac, −14%), au niveau du prix budgété Q4 (17 678).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>NOTE: Prix du soja en septembre 2026: 23 879 FCFA/sac (hausse de +2 000 XAF/sac depuis le 23/07/2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>Ratio global: 4.7:1 (vs 3.3:1 le 30/09).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="14" t="inlineStr">
-        <is>
-          <t>Note: T2/T3 portent sur le 03/10 (dernier jour avec commandes Livrées; le 04/10 est un dimanche et le 05/10 n'a pas encore de commandes Livrées à l'extraction). Comparaison vs 30/09 (bilan septembre complet).</t>
+          <t>Ratio global: 2.3:1 (vs 3.3:1 le 30/09).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Note: T2/T3 portent sur le 10/10 (dernier jour avec commandes Livrées; le 11/10 est un dimanche). Comparaison vs 30/09 (bilan septembre complet).</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1983,7 +1947,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TABLEAU 3 - SOJA sans concentres le 03/10/2026</t>
+          <t>TABLEAU 3 - SOJA sans concentres le 10/10/2026</t>
         </is>
       </c>
     </row>
@@ -2047,29 +2011,29 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139838</t>
+          <t>SO2610-141809</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>CU2410-01130 -  SEPTENTRION VETERINAIRE SARL</t>
+          <t>CU2407-00759 -  MATENNE MBA CHANTAL OLGA</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Ndobo</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1120</v>
+        <v>100</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -2088,12 +2052,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139805</t>
+          <t>SO2610-141788</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>CU2606-14515 -  LANBOU TINO</t>
+          <t>CU2507-13426 -  ZANGHO WILFRIED</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2107,10 +2071,10 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -2129,29 +2093,29 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139898</t>
+          <t>SO2610-141972</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>CU2407-00601 -  FOKO</t>
+          <t>CU2407-00412 -  WANDJA JEAN CLAUDE</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Famla</t>
+          <t>Buea</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -2170,12 +2134,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139786</t>
+          <t>SO2610-141960</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>CU2504-13345 -  STE K'MDEU FARMS SARL (PEUMENI PASCAL)</t>
+          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2189,10 +2153,10 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
@@ -2211,29 +2175,29 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139893</t>
+          <t>SO2610-141902</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>ZOCL00002000 -  KUHLIFARM COOP-BOD (KUHLIFARM COOP-BOD)</t>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Nkongsamba</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -2252,29 +2216,29 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139910</t>
+          <t>SO2610-141910</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
@@ -2293,29 +2257,29 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139970</t>
+          <t>SO2610-141812</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -2334,29 +2298,29 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139799</t>
+          <t>SO2610-141814</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
@@ -2375,22 +2339,22 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139756</t>
+          <t>SO2610-141904</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
+          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Famla</t>
+          <t>Pk11</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
@@ -2416,17 +2380,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139832</t>
+          <t>SO2610-141903</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
+          <t>CU2407-00140 -  CLIENTS COMPTOIR BAF-DJELENG</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Famla</t>
+          <t>Djeleng</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -2457,17 +2421,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139853</t>
+          <t>SO2610-141779</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00004 -  CLIENT COMPTOIR AXE LOURD</t>
+          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Village</t>
+          <t>Pk11</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -2476,10 +2440,10 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -2498,29 +2462,29 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139925</t>
+          <t>SO2610-141819</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
@@ -2539,29 +2503,29 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139971</t>
+          <t>SO2610-141896</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>CU2407-00148 -  CLIENTS COMPTOIR NKOABANG</t>
+          <t>CU2407-00140 -  CLIENTS COMPTOIR BAF-DJELENG</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Nkoabang</t>
+          <t>Djeleng</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -2580,29 +2544,29 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>SO2610-139791</t>
+          <t>SO2610-141986</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>CU2407-00149 -  CLIENTS COMPTOIR NKOLBISSON</t>
+          <t>CU2406-00076 -  CLIENTS COMPTOIR BUEA</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Nkolbisson</t>
+          <t>Buea</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
@@ -2616,402 +2580,33 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>SO2610-139784</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Famla</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Ouest</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Livrée</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>SO2610-139808</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>CU2508-13471 -  TCHEDING MIKE MARIE</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Nkolbisson</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Centre</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Livrée</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>184</v>
+      </c>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>SO2610-139826</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>CU2406-00004 -  CLIENT COMPTOIR AXE LOURD</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Village</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Littoral</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Livrée</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Total soja-only: 14 cmdes (9.2 t) le 10/10/2026</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>SO2610-139867</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Famla</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Ouest</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Livrée</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>SO2610-139868</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>CU2407-00148 -  CLIENTS COMPTOIR NKOABANG</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Nkoabang</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Centre</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>Livrée</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>SO2610-139892</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>CU2406-00004 -  CLIENT COMPTOIR AXE LOURD</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Village</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Littoral</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Livrée</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>SO2610-139949</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Famla</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Ouest</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G25" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>Livrée</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>SO2610-139967</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Famla</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Ouest</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>Livrée</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>SO2610-139914</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>CU2407-00175 -  CLIENT COMPTOIR NKONGSSAMBA</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Nkongsamba</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>Littoral</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>Livrée</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="n"/>
-      <c r="B28" s="8" t="n"/>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="n"/>
-      <c r="E28" s="8" t="n"/>
-      <c r="F28" s="8" t="n">
-        <v>66.90000000000001</v>
-      </c>
-      <c r="G28" s="8" t="n">
-        <v>1337</v>
-      </c>
-      <c r="H28" s="8" t="n"/>
-      <c r="I28" s="8" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>Total soja-only: 23 cmdes (66.9 t) le 03/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Precedent (30/09): 38 cmdes (79.3 t)</t>
         </is>
@@ -3046,7 +2641,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Aucune mesure de stock physique fournie depuis le 08/08/2026 (magasins centraux BEKOKO). La date de rupture ne peut pas etre recalculee. Mise a jour 05/10/2026.</t>
+          <t>Aucune mesure de stock physique fournie depuis le 08/08/2026 (magasins centraux BEKOKO). La date de rupture ne peut pas etre recalculee. Mise a jour 10/10/2026.</t>
         </is>
       </c>
     </row>
@@ -3177,12 +2772,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>610.6 t</t>
+          <t>2451.1 t</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>01-03/10 (rien de Livré le 04-05/10)</t>
+          <t>01-10/10 (Livrée)</t>
         </is>
       </c>
     </row>
@@ -3194,24 +2789,24 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>171.6 t</t>
+          <t>693.1 t</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>01-03/10 (rien de Livré le 04-05/10)</t>
+          <t>01-10/10 (Livrée)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>ANALYSE: Sans nouvelle mesure de stock physique, la projection de rupture (methode BEKOKO: stock net - consommation hebdomadaire) ne peut pas etre actualisee pour octobre.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Action: demander une mesure physique des magasins centraux BEKOKO (formats 50/1/5/25 kg) pour relancer le calcul.</t>
         </is>
@@ -3228,7 +2823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3250,7 +2845,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Données Livrées au 05/10/2026. Jours ouvrés (lun-sam) en couleur, dimanches en gris.</t>
+          <t>Données Livrées au 10/10/2026. Jours ouvrés (lun-sam) en couleur, dimanches en gris.</t>
         </is>
       </c>
     </row>
@@ -3306,18 +2901,18 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>222.3</v>
+        <v>224.3</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>69</v>
+        <v>69.2</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>3.22:1</t>
+          <t>3.24:1</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>3.22</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="6">
@@ -3335,18 +2930,18 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>223.5</v>
+        <v>311.1</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>67.3</v>
+        <v>84.7</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>3.32:1</t>
+          <t>3.67:1</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>3.32</v>
+        <v>3.67</v>
       </c>
     </row>
     <row r="7">
@@ -3364,41 +2959,41 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>164.9</v>
+        <v>247.6</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>35.2</v>
+        <v>52.1</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>4.69:1</t>
+          <t>4.76:1</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>4.69</v>
+        <v>4.76</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>04/10/2026</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Dim</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="15" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3419,56 +3014,204 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0</v>
+        <v>349.1</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0</v>
+        <v>124.5</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>2.8:1</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>327.7</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>3.4:1</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Mer</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>269.3</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>3.11:1</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>3.11</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Jeu</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>412.8</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>6.07:1</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>6.07</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Ven</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>219.8</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>3.0:1</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>2.33:1</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>2.33</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>NOTES DE LECTURE:</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>• La ligne "Soja" (bleu) montre la consommation journalière de tourteaux de soja (prix de référence: 23 879 FCFA/sac en septembre 2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>• La ligne "Soja" (bleu) montre la consommation journalière de tourteaux de soja (prix de référence: 23 879 FCFA/sac en septembre 2026 ; 19 318 FCFA/sac en moyenne octobre MTD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>• La ligne "Concentrés" (or) montre la consommation journalière de concentrés (BELGO Chair/Ponte/Porc).</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>• Le ratio soja:conc cible est 3:1 (objectif bundle). Un ratio supérieur signifie que les clients achètent plus de soja que de concentrés — dégradation du bundle.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>• Les dimanches sont grisés (pas de ventes). Octobre est un mois en cours (MTD au 05/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>• À observer: la tendance soja/concentrés en début octobre vs septembre — le ratio doit rester proche de 3:1.</t>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>• Les dimanches sont grisés (pas de ventes). Octobre est un mois en cours (MTD au 10/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>• À observer: après la baisse du 07/10 (20 500 → 17 600 FCFA/sac, −14%), la reprise soja se confirme-t-elle sans dégrader le ratio 3:1 ?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour octobre MTD au 17/10 (extraction 67) : performance mensuelle, zéro achat (section 5.4 MTD, seuil ≤ 17j), bundle soja-concentrés (section 10 MTD), analyse trend (P2 12-17/10, 5 semaines, effet 2e baisse confirmé), booster 13 mois, soja octobre (T1-T5)
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/download/analyse_soja_octobre.xlsx
+++ b/download/analyse_soja_octobre.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="T1 - Moy jour soja par agence" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="T2 - Commandes soja 10-10" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="T3 - Soja-only 10-10" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="T2 - Commandes soja 17-10" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="T3 - Soja-only 17-10" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="T4 - Stock soja et rupture" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="T5 - Tendance Octobre" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,10 @@
     <font>
       <i val="1"/>
       <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="009C0006"/>
       <sz val="10"/>
     </font>
     <font>
@@ -157,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -166,16 +170,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -300,12 +305,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$A$5:$A$14</f>
+              <f>'T5 - Tendance Octobre'!$A$5:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$D$5:$D$14</f>
+              <f>'T5 - Tendance Octobre'!$D$5:$D$21</f>
             </numRef>
           </val>
         </ser>
@@ -335,12 +340,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$A$5:$A$14</f>
+              <f>'T5 - Tendance Octobre'!$A$5:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$E$5:$E$14</f>
+              <f>'T5 - Tendance Octobre'!$E$5:$E$21</f>
             </numRef>
           </val>
         </ser>
@@ -447,12 +452,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$A$5:$A$14</f>
+              <f>'T5 - Tendance Octobre'!$A$5:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'T5 - Tendance Octobre'!$G$5:$G$14</f>
+              <f>'T5 - Tendance Octobre'!$G$5:$G$21</f>
             </numRef>
           </val>
         </ser>
@@ -877,7 +882,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>01/10 au 10/10/2026 (9j). Livree. lun-sam. Mise a jour 10/10/2026.</t>
+          <t>01/10 au 17/10/2026 (15j). Livree. lun-sam. Mise a jour 17/10/2026.</t>
         </is>
       </c>
     </row>
@@ -920,14 +925,14 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>710.4</v>
+        <v>1190.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>78.90000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>+27.5 t/j</t>
+          <t>+28.0 t/j</t>
         </is>
       </c>
     </row>
@@ -943,14 +948,14 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>362.3</v>
+        <v>567.7</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>40.3</v>
+        <v>37.8</v>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>+18.8 t/j</t>
+          <t>+16.4 t/j</t>
         </is>
       </c>
     </row>
@@ -966,14 +971,14 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>283.1</v>
+        <v>416.4</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>31.5</v>
+        <v>27.8</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>+15.3 t/j</t>
+          <t>+11.6 t/j</t>
         </is>
       </c>
     </row>
@@ -989,106 +994,106 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>194</v>
+        <v>338</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>21.6</v>
+        <v>22.5</v>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>+6.4 t/j</t>
+          <t>+7.3 t/j</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Village</t>
+          <t>Ahala</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>122.5</v>
+        <v>228.2</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>13.6</v>
+        <v>15.2</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+1.9 t/j</t>
+          <t>+4.7 t/j</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Ahala</t>
+          <t>Mbouda</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>117.3</v>
+        <v>220</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>13</v>
+        <v>14.7</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>+2.6 t/j</t>
+          <t>+6.3 t/j</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Nkoabang</t>
+          <t>Village</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>115.3</v>
+        <v>199.5</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>12.8</v>
+        <v>13.3</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>+2.6 t/j</t>
+          <t>+1.5 t/j</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Mbouda</t>
+          <t>Nkoabang</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>113</v>
+        <v>192</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>12.6</v>
+        <v>12.8</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>+4.2 t/j</t>
+          <t>+2.6 t/j</t>
         </is>
       </c>
     </row>
@@ -1104,60 +1109,60 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>99</v>
+        <v>184.5</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>11</v>
+        <v>12.3</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>+2.2 t/j</t>
+          <t>+3.5 t/j</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Nkongsamba</t>
+          <t>Bertoua</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>96</v>
+        <v>159.2</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>+4.1 t/j</t>
+          <t>+2.7 t/j</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Bertoua</t>
+          <t>Nkongsamba</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>90.90000000000001</v>
+        <v>133.2</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>10.1</v>
+        <v>8.9</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>+2.2 t/j</t>
+          <t>+2.3 t/j</t>
         </is>
       </c>
     </row>
@@ -1173,14 +1178,14 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>67.5</v>
+        <v>125.2</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>7.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>+1.6 t/j</t>
+          <t>+2.5 t/j</t>
         </is>
       </c>
     </row>
@@ -1196,14 +1201,14 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>47.1</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>5.2</v>
+        <v>5.8</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>+2.8 t/j</t>
+          <t>+3.3 t/j</t>
         </is>
       </c>
     </row>
@@ -1219,14 +1224,14 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>30.8</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>3.4</v>
+        <v>4.5</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+1.1 t/j</t>
+          <t>+2.2 t/j</t>
         </is>
       </c>
     </row>
@@ -1242,104 +1247,104 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>0.2</v>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>-0.1 t/j</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>TOTAL Ouest</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Ouest</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n">
-        <v>1106.4</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>122.9</v>
-      </c>
-      <c r="E20" s="6" t="n"/>
+      <c r="C20" s="7" t="n">
+        <v>1826.9</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>121.8</v>
+      </c>
+      <c r="E20" s="7" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>TOTAL Centre</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Centre</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
-        <v>595.4</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>66.2</v>
-      </c>
-      <c r="E21" s="6" t="n"/>
+      <c r="C21" s="7" t="n">
+        <v>1071</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="E21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>TOTAL Littoral</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Littoral</t>
         </is>
       </c>
-      <c r="C22" s="6" t="n">
-        <v>747.3</v>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>83</v>
-      </c>
-      <c r="E22" s="6" t="n"/>
+      <c r="C22" s="7" t="n">
+        <v>1210</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>80.7</v>
+      </c>
+      <c r="E22" s="7" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n">
-        <v>2451.1</v>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>272.3</v>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>+93.1 t/j vs 179.3</t>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n">
+        <v>4110.9</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>274.1</v>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>+94.8 t/j vs 179.3</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>NOTE: Prix du soja en septembre 2026: 23 879 FCFA/sac (hausse de +2 000 XAF/sac depuis le 23/07/2026).</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>Moyenne/jour globale: 272.3 t/j (5446 sacs) sur 9j.</t>
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Moyenne/jour globale: 274.1 t/j (5481 sacs) sur 15j.</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1358,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Note: extraction du 12/10 — commandes Livrées jusqu'au 10/10 (le 11/10 est un dimanche).</t>
+          <t>Note: extraction du 19/10 — commandes Livrées jusqu'au 17/10 (le 18/10 est un dimanche).</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1383,14 +1388,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TABLEAU 2 - Commandes SOJA le 10/10/2026 par agence</t>
+          <t>TABLEAU 2 - Commandes SOJA le 17/10/2026 par agence</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Livree. Ratio en sacs 50kg-equivalent. Mise a jour 10/10/2026.</t>
+          <t>Livree. Ratio en sacs 50kg-equivalent. Mise a jour 17/10/2026.</t>
         </is>
       </c>
     </row>
@@ -1443,82 +1448,82 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>3.9:1</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>-17 cmdes</t>
+          <t>4.4:1</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>-16 cmdes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Messassi</t>
+          <t>Mbouda</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>2.6:1</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>-2 cmdes</t>
+          <t>2.3:1</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>+6 cmdes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Bertoua</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="D7" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="E7" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1.7:1</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
+          <t>1.6:1</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>-6 cmdes</t>
         </is>
@@ -1539,17 +1544,17 @@
         <v>10</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>3.2:1</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
+          <t>2.9:1</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>+4 cmdes</t>
         </is>
@@ -1558,31 +1563,31 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Mbouda</t>
+          <t>Nkoabang</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>1.3:1</t>
+          <t>4.4:1</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>+2 cmdes</t>
+          <t>-1 cmdes</t>
         </is>
       </c>
     </row>
@@ -1598,29 +1603,29 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>2.8:1</t>
+          <t>5.6:1</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>+2 cmdes</t>
+          <t>-1 cmdes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Bertoua</t>
+          <t>Ahala</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1629,293 +1634,231 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>1.2:1</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>-11 cmdes</t>
+          <t>3.3:1</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>-7 cmdes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Ahala</t>
+          <t>Pk11</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>2.5:1</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>-6 cmdes</t>
+          <t>3.0:1</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>-12 cmdes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Djeleng</t>
+          <t>Village</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>2.6:1</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>-9 cmdes</t>
+          <t>0.2:1</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>-13 cmdes</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Nkoabang</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Centre</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>3.6:1</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>-3 cmdes</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Nkongsamba</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Littoral</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>1.5:1</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>-6 cmdes</t>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>2.8:1</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>-109 cmdes vs 195</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n">
-        <v>111</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>97</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>2.3:1</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>-84 cmdes vs 195</t>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Distribution ratios (bundle seulement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Tranche</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Nb cmdes</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Part</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Distribution ratios (bundle seulement)</t>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>&lt;= 3:1</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>73%</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Tranche</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Nb cmdes</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Part</t>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>3-5:1</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>15%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>&lt;= 3:1</t>
+          <t>5-10:1</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>77%</t>
+          <t>11%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>3-5:1</t>
+          <t>10-20:1</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>2%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>5-10:1</t>
+          <t>&gt; 20:1</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>10-20:1</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>&gt; 20:1</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
           <t>0%</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>NOTE: Prix du soja: 23 879 FCFA/sac en moyenne septembre 2026 ; octobre MTD 19 318 FCFA/sac — baisse du 07/10 (20 500 → 17 600 FCFA/sac, −14%), au niveau du prix budgété Q4 (17 678).</t>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>NOTE: Prix du soja: 23 879 FCFA/sac en moyenne septembre 2026 ; octobre MTD 18 654 FCFA/sac — baisse du 07/10 (20 500 → 17 600 FCFA/sac, −14%), au niveau du prix budgété Q4 (17 678).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Ratio global: 2.8:1 (vs 3.3:1 le 30/09).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>Ratio global: 2.3:1 (vs 3.3:1 le 30/09).</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>Note: T2/T3 portent sur le 10/10 (dernier jour avec commandes Livrées; le 11/10 est un dimanche). Comparaison vs 30/09 (bilan septembre complet).</t>
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Note: T2/T3 portent sur le 17/10 (dernier jour avec commandes Livrées; le 18/10 est un dimanche). Comparaison vs 30/09 (bilan septembre complet).</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1947,7 +1890,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TABLEAU 3 - SOJA sans concentres le 10/10/2026</t>
+          <t>TABLEAU 3 - SOJA sans concentres le 17/10/2026</t>
         </is>
       </c>
     </row>
@@ -2011,12 +1954,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141809</t>
+          <t>SO2610-143906</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>CU2407-00759 -  MATENNE MBA CHANTAL OLGA</t>
+          <t>CU2407-00794 -  PENKA DEFFO DANIEL</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2030,10 +1973,10 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -2052,29 +1995,29 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141788</t>
+          <t>SO2610-144093</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>CU2507-13426 -  ZANGHO WILFRIED</t>
+          <t>CU2410-01118 -  PROVENDERIE LA REFERENCE</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Famla</t>
+          <t>Nkoabang</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -2093,29 +2036,29 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141972</t>
+          <t>SO2610-143902</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>CU2407-00412 -  WANDJA JEAN CLAUDE</t>
+          <t>CU2407-00926 -  SANLAI SARL</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Buea</t>
+          <t>Nkolbisson</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -2134,29 +2077,29 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141960</t>
+          <t>SO2610-144034</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
+          <t>CU2502-01218 -  AWAMBA FABRICE (KEOGUE TCHINDA)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Ahala</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.3</v>
+        <v>1.5</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
@@ -2175,12 +2118,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141902</t>
+          <t>SO2610-143877</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
+          <t>CU2607-14567 -  TALLA WAFFEU MAURICE</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -2194,10 +2137,10 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.2</v>
+        <v>1.4</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -2216,12 +2159,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141910</t>
+          <t>SO2610-143869</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
+          <t>CU2601-14332 -  KENMOGNE GASTON</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -2235,10 +2178,10 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.15</v>
+        <v>1.35</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
@@ -2257,29 +2200,29 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141812</t>
+          <t>SO2610-144086</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
+          <t>CU2407-00445 -  MOUGET EVARISTUS ACHU</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Famla</t>
+          <t>Buea</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Littoral</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -2298,7 +2241,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141814</t>
+          <t>SO2610-143878</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -2317,10 +2260,10 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
@@ -2339,29 +2282,29 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141904</t>
+          <t>SO2610-143984</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -2380,17 +2323,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141903</t>
+          <t>SO2610-143998</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>CU2407-00140 -  CLIENTS COMPTOIR BAF-DJELENG</t>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Djeleng</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -2399,10 +2342,10 @@
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
@@ -2421,29 +2364,29 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141779</t>
+          <t>SO2610-144006</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Pk11</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Littoral</t>
+          <t>Ouest</t>
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -2462,29 +2405,29 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141819</t>
+          <t>SO2610-144060</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
+          <t>CU2407-00149 -  CLIENTS COMPTOIR NKOLBISSON</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Famla</t>
+          <t>Nkolbisson</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Ouest</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
@@ -2503,17 +2446,17 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141896</t>
+          <t>SO2610-143947</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>CU2407-00140 -  CLIENTS COMPTOIR BAF-DJELENG</t>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Djeleng</t>
+          <t>Famla</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -2522,10 +2465,10 @@
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -2544,69 +2487,315 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>SO2610-141986</t>
+          <t>SO2610-144074</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>CU2406-00076 -  CLIENTS COMPTOIR BUEA</t>
+          <t>CU2407-00148 -  CLIENTS COMPTOIR NKOABANG</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Buea</t>
+          <t>Nkoabang</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Livrée</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>SO2610-143890</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Famla</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Ouest</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Livrée</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>SO2610-143910</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>CU2407-00143 -  CLIENTS COMPTOIR BERTOUA</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Bertoua</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Livrée</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>SO2610-143898</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>CU2406-00122 -  CLIENTS COMPTOIR FAMLA</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Famla</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Ouest</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Livrée</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>SO2610-143930</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>CU2407-00148 -  CLIENTS COMPTOIR NKOABANG</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Nkoabang</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Livrée</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>SO2610-144004</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>CU2407-00143 -  CLIENTS COMPTOIR BERTOUA</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Bertoua</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Livrée</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>SO2610-143936</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>CU2406-00012 -  CLIENTS COMPTOIR PK11</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Pk11</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
           <t>Littoral</t>
         </is>
       </c>
-      <c r="F18" s="4" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G18" s="4" t="n">
+      <c r="F24" s="4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G24" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Livrée</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="G19" s="7" t="n">
-        <v>184</v>
-      </c>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="7" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>Total soja-only: 14 cmdes (9.2 t) le 10/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>290</v>
+      </c>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Total soja-only: 20 cmdes (14.5 t) le 17/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Precedent (30/09): 38 cmdes (79.3 t)</t>
         </is>
@@ -2641,7 +2830,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Aucune mesure de stock physique fournie depuis le 08/08/2026 (magasins centraux BEKOKO). La date de rupture ne peut pas etre recalculee. Mise a jour 10/10/2026.</t>
+          <t>Aucune mesure de stock physique fournie depuis le 08/08/2026 (magasins centraux BEKOKO). La date de rupture ne peut pas etre recalculee. Mise a jour 17/10/2026.</t>
         </is>
       </c>
     </row>
@@ -2772,12 +2961,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>2451.1 t</t>
+          <t>4110.9 t</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>01-10/10 (Livrée)</t>
+          <t>01-17/10 (Livrée)</t>
         </is>
       </c>
     </row>
@@ -2789,24 +2978,24 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>693.1 t</t>
+          <t>1249.6 t</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>01-10/10 (Livrée)</t>
+          <t>01-17/10 (Livrée)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>ANALYSE: Sans nouvelle mesure de stock physique, la projection de rupture (methode BEKOKO: stock net - consommation hebdomadaire) ne peut pas etre actualisee pour octobre.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Action: demander une mesure physique des magasins centraux BEKOKO (formats 50/1/5/25 kg) pour relancer le calcul.</t>
         </is>
@@ -2823,7 +3012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2845,7 +3034,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Données Livrées au 10/10/2026. Jours ouvrés (lun-sam) en couleur, dimanches en gris.</t>
+          <t>Données Livrées au 17/10/2026. Jours ouvrés (lun-sam) en couleur, dimanches en gris.</t>
         </is>
       </c>
     </row>
@@ -2930,18 +3119,18 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>311.1</v>
+        <v>353.6</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>84.7</v>
+        <v>90.8</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>3.67:1</t>
+          <t>3.89:1</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>3.67</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="7">
@@ -2959,41 +3148,41 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>247.6</v>
+        <v>249.6</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>52.1</v>
+        <v>53.1</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>4.76:1</t>
+          <t>4.7:1</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>4.76</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>04/10/2026</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Dim</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3014,18 +3203,18 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>349.1</v>
+        <v>366.6</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>124.5</v>
+        <v>129.5</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2.8:1</t>
+          <t>2.83:1</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2.8</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="10">
@@ -3043,18 +3232,18 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>327.7</v>
+        <v>332.7</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>96.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>3.4:1</t>
+          <t>3.43:1</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>3.4</v>
+        <v>3.43</v>
       </c>
     </row>
     <row r="11">
@@ -3072,18 +3261,18 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>269.3</v>
+        <v>299.9</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>86.7</v>
+        <v>88</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>3.11:1</t>
+          <t>3.41:1</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>3.11</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="12">
@@ -3101,18 +3290,18 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>412.8</v>
+        <v>448.3</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>68</v>
+        <v>87.8</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>6.07:1</t>
+          <t>5.11:1</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>6.07</v>
+        <v>5.11</v>
       </c>
     </row>
     <row r="13">
@@ -3130,18 +3319,18 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>219.8</v>
+        <v>277.3</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>73.2</v>
+        <v>96.3</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>3.0:1</t>
+          <t>2.88:1</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>2.88</v>
       </c>
     </row>
     <row r="14">
@@ -3159,57 +3348,257 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>89.40000000000001</v>
+        <v>169.8</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>38.3</v>
+        <v>52.2</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>2.33:1</t>
+          <t>3.26:1</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2.33</v>
+        <v>3.26</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>11/10/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Dim</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>391.4</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>2.61:1</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>271.7</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>2.88:1</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>2.88</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Mer</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>221.9</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>85.3</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>2.6:1</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Jeu</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>200.8</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>3.33:1</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Ven</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>198.5</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>3.41:1</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>3.41</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>2.78:1</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>NOTES DE LECTURE:</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>• La ligne "Soja" (bleu) montre la consommation journalière de tourteaux de soja (prix de référence: 23 879 FCFA/sac en septembre 2026 ; 19 318 FCFA/sac en moyenne octobre MTD).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>• La ligne "Soja" (bleu) montre la consommation journalière de tourteaux de soja (prix de référence: 23 879 FCFA/sac en septembre 2026 ; 18 654 FCFA/sac en moyenne octobre MTD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>• La ligne "Concentrés" (or) montre la consommation journalière de concentrés (BELGO Chair/Ponte/Porc).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>• Le ratio soja:conc cible est 3:1 (objectif bundle). Un ratio supérieur signifie que les clients achètent plus de soja que de concentrés — dégradation du bundle.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>• Les dimanches sont grisés (pas de ventes). Octobre est un mois en cours (MTD au 10/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>• Les dimanches sont grisés (pas de ventes). Octobre est un mois en cours (MTD au 17/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>• À observer: après la baisse du 07/10 (20 500 → 17 600 FCFA/sac, −14%), la reprise soja se confirme-t-elle sans dégrader le ratio 3:1 ?</t>
         </is>

</xml_diff>